<commit_message>
modifying docker compose and adding planned tools
</commit_message>
<xml_diff>
--- a/checkboxes.xlsx
+++ b/checkboxes.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9285" windowHeight="3690"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>WSL2</t>
   </si>
@@ -34,23 +34,60 @@
     <t>DBeaver</t>
   </si>
   <si>
-    <t>PostgreSQL (Star Schemas)</t>
-  </si>
-  <si>
     <t>Docker (Avoid Dependency Hell)</t>
   </si>
   <si>
     <t>GitHub Actions (CI/CD)</t>
+  </si>
+  <si>
+    <t>Synthea</t>
+  </si>
+  <si>
+    <t>Java</t>
+  </si>
+  <si>
+    <t>GCP</t>
+  </si>
+  <si>
+    <t>DuckDB</t>
+  </si>
+  <si>
+    <t>PostgreSQL</t>
+  </si>
+  <si>
+    <t>Terraform</t>
+  </si>
+  <si>
+    <t>Google AI Studio (RAG)</t>
+  </si>
+  <si>
+    <t>Nextflow</t>
+  </si>
+  <si>
+    <t>pgvector</t>
+  </si>
+  <si>
+    <t>LangGraph</t>
+  </si>
+  <si>
+    <t>Epigenetic Clock Algorithm Implementation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -71,24 +108,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -111,17 +148,47 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,95 +493,134 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="27.5703125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="5"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="6"/>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="7"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="7"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7"/>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5"/>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="6"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="7"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="5"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="5"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="5"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="5"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="B10" s="7"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="5"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+      <c r="B11" s="7"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+      <c r="A12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="7"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+      <c r="A13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="7"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+      <c r="A14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="7"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
+      <c r="A15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B16" s="3"/>
+      <c r="A16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="7"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="7"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
basic updates. still troubleshooting
</commit_message>
<xml_diff>
--- a/checkboxes.xlsx
+++ b/checkboxes.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="9285" windowHeight="3690"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>WSL2</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t>Epigenetic Clock Algorithm Implementation</t>
+  </si>
+  <si>
+    <t>GDPR Compliance</t>
   </si>
 </sst>
 </file>
@@ -493,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.42578125" style="1" customWidth="1"/>
@@ -616,8 +619,14 @@
       <c r="B19" s="7"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+      <c r="A20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>